<commit_message>
Changes related to contact POM, Logging, Account scenarios
</commit_message>
<xml_diff>
--- a/tests/test-data/TestData.xlsx
+++ b/tests/test-data/TestData.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Neha\TrailblazersCRM\tests\test-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Neha\SuiteCRM_PAT\tests\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11835" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11835"/>
   </bookViews>
   <sheets>
     <sheet name="Accounts" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="66">
   <si>
     <t>AccountName</t>
   </si>
@@ -192,15 +192,6 @@
     <t>Third Test account creation.</t>
   </si>
   <si>
-    <t>Name field validation.</t>
-  </si>
-  <si>
-    <t>validation@test</t>
-  </si>
-  <si>
-    <t>Incorrect email validation.</t>
-  </si>
-  <si>
     <t>TestCase</t>
   </si>
   <si>
@@ -223,12 +214,6 @@
   </si>
   <si>
     <t>TC004</t>
-  </si>
-  <si>
-    <t>TC005</t>
-  </si>
-  <si>
-    <t>TC006</t>
   </si>
   <si>
     <t>ExpectedResult</t>
@@ -244,7 +229,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -255,14 +240,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -311,17 +288,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -329,8 +304,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -631,7 +605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -655,7 +629,7 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -702,13 +676,13 @@
       <c r="P1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="5" t="s">
-        <v>68</v>
+      <c r="Q1" s="4" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>15</v>
@@ -761,7 +735,7 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>27</v>
@@ -807,11 +781,14 @@
       </c>
       <c r="P3" s="1" t="s">
         <v>53</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>35</v>
@@ -857,11 +834,14 @@
       </c>
       <c r="P4" s="1" t="s">
         <v>54</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>44</v>
@@ -906,111 +886,13 @@
       <c r="P5" s="1" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B7" s="1" t="s">
+      <c r="Q5" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="P7" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D7" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1025,25 +907,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>68</v>
+      <c r="A1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1062,25 +944,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B1" s="4" t="s">
+      <c r="A1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>60</v>
+      <c r="C1" s="3" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>62</v>
-      </c>
       <c r="C2" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>